<commit_message>
Added few Test Cases in IWP-Demo
</commit_message>
<xml_diff>
--- a/KatalonData/IWPBootstrapDataDemo/VRelayPaymentsCC_23.xlsx
+++ b/KatalonData/IWPBootstrapDataDemo/VRelayPaymentsCC_23.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t476046\Documents\VPS-Katalon-feature-VRelay\KatalonData\IWPBootstrapDataDemo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2998B799-21D3-4B71-87BC-DEA04B05A838}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B00462BE-1E37-4E34-A06D-503319B81234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="1752" windowWidth="17280" windowHeight="9972" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2844" yWindow="2052" windowWidth="17280" windowHeight="9972" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PayNowCCNoCF" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="PayNowDCNoCF" sheetId="4" r:id="rId4"/>
     <sheet name="PayNowDCSCF" sheetId="5" r:id="rId5"/>
     <sheet name="PayNowDCDCF" sheetId="6" r:id="rId6"/>
+    <sheet name="NoModifyAmountCC" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="33">
   <si>
     <t>Result</t>
   </si>
@@ -126,6 +127,9 @@
   </si>
   <si>
     <t>Fri Jun 12 19:34:19 IST 2026</t>
+  </si>
+  <si>
+    <t>Pay Now Credit Card, Emulator Data is overwritten</t>
   </si>
 </sst>
 </file>
@@ -1005,4 +1009,90 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD268279-6E23-4C76-967B-33DCA119E4A1}">
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="C2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2">
+        <v>35</v>
+      </c>
+      <c r="F2">
+        <v>6425</v>
+      </c>
+      <c r="G2">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="I2">
+        <v>2</v>
+      </c>
+      <c r="J2">
+        <v>5</v>
+      </c>
+      <c r="K2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>3</v>
+      </c>
+      <c r="N2">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>